<commit_message>
Duties: Standardize all duty names to official full names across master JSON and Excel
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
@@ -570,7 +570,7 @@
         <v>ชาย</v>
       </c>
       <c r="I5" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -605,7 +605,7 @@
         <v>หญิง</v>
       </c>
       <c r="I6" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -640,7 +640,7 @@
         <v>หญิง</v>
       </c>
       <c r="I7" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -675,7 +675,7 @@
         <v>หญิง</v>
       </c>
       <c r="I8" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -710,7 +710,7 @@
         <v>ชาย</v>
       </c>
       <c r="I9" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -745,7 +745,7 @@
         <v>ชาย</v>
       </c>
       <c r="I10" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -780,7 +780,7 @@
         <v>ชาย</v>
       </c>
       <c r="I11" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -815,7 +815,7 @@
         <v>ชาย</v>
       </c>
       <c r="I12" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -850,7 +850,7 @@
         <v>หญิง</v>
       </c>
       <c r="I13" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -885,7 +885,7 @@
         <v>หญิง</v>
       </c>
       <c r="I14" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -920,7 +920,7 @@
         <v>หญิง</v>
       </c>
       <c r="I15" t="str">
-        <v>ฟุตบอล, สแตนเชียร์</v>
+        <v>ฟุตบอล, ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J15" t="str">
         <v>085-226-6457</v>
@@ -955,7 +955,7 @@
         <v>ชาย</v>
       </c>
       <c r="I16" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -990,7 +990,7 @@
         <v>ชาย</v>
       </c>
       <c r="I17" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1025,7 +1025,7 @@
         <v>หญิง</v>
       </c>
       <c r="I18" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1060,7 +1060,7 @@
         <v>หญิง</v>
       </c>
       <c r="I19" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1095,7 +1095,7 @@
         <v>หญิง</v>
       </c>
       <c r="I20" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J20" t="str">
         <v/>
@@ -1130,7 +1130,7 @@
         <v>หญิง</v>
       </c>
       <c r="I21" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J21" t="str">
         <v/>
@@ -1165,7 +1165,7 @@
         <v>ชาย</v>
       </c>
       <c r="I22" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J22" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>ชาย</v>
       </c>
       <c r="I23" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J23" t="str">
         <v/>
@@ -1235,7 +1235,7 @@
         <v>ชาย</v>
       </c>
       <c r="I24" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J24" t="str">
         <v/>
@@ -1270,7 +1270,7 @@
         <v>ชาย</v>
       </c>
       <c r="I25" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J25" t="str">
         <v/>
@@ -1305,7 +1305,7 @@
         <v>หญิง</v>
       </c>
       <c r="I26" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -1340,7 +1340,7 @@
         <v>หญิง</v>
       </c>
       <c r="I27" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J27" t="str">
         <v/>
@@ -1375,7 +1375,7 @@
         <v>หญิง</v>
       </c>
       <c r="I28" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J28" t="str">
         <v/>
@@ -1410,7 +1410,7 @@
         <v>ชาย</v>
       </c>
       <c r="I29" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -1445,7 +1445,7 @@
         <v>ชาย</v>
       </c>
       <c r="I30" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J30" t="str">
         <v/>
@@ -1480,7 +1480,7 @@
         <v>ชาย</v>
       </c>
       <c r="I31" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J31" t="str">
         <v/>
@@ -1515,7 +1515,7 @@
         <v>หญิง</v>
       </c>
       <c r="I32" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J32" t="str">
         <v/>
@@ -1550,7 +1550,7 @@
         <v>หญิง</v>
       </c>
       <c r="I33" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J33" t="str">
         <v/>
@@ -1585,7 +1585,7 @@
         <v>หญิง</v>
       </c>
       <c r="I34" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J34" t="str">
         <v/>
@@ -1620,7 +1620,7 @@
         <v>หญิง</v>
       </c>
       <c r="I35" t="str">
-        <v>วอลเลย์บอล, สแตนเชียร์</v>
+        <v>วอลเลย์บอล, ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J35" t="str">
         <v/>
@@ -1655,7 +1655,7 @@
         <v>ชาย</v>
       </c>
       <c r="I36" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -1690,7 +1690,7 @@
         <v>ชาย</v>
       </c>
       <c r="I37" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J37" t="str">
         <v/>
@@ -1725,7 +1725,7 @@
         <v>ชาย</v>
       </c>
       <c r="I38" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J38" t="str">
         <v/>
@@ -1760,7 +1760,7 @@
         <v>ชาย</v>
       </c>
       <c r="I39" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J39" t="str">
         <v/>
@@ -1795,7 +1795,7 @@
         <v>หญิง</v>
       </c>
       <c r="I40" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J40" t="str">
         <v/>
@@ -1830,7 +1830,7 @@
         <v>หญิง</v>
       </c>
       <c r="I41" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -1865,7 +1865,7 @@
         <v>หญิง</v>
       </c>
       <c r="I42" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J42" t="str">
         <v/>
@@ -1900,7 +1900,7 @@
         <v>ชาย</v>
       </c>
       <c r="I43" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J43" t="str">
         <v/>
@@ -1935,7 +1935,7 @@
         <v>ชาย</v>
       </c>
       <c r="I44" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J44" t="str">
         <v/>
@@ -1970,7 +1970,7 @@
         <v>ชาย</v>
       </c>
       <c r="I45" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -2005,7 +2005,7 @@
         <v>หญิง</v>
       </c>
       <c r="I46" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J46" t="str">
         <v/>
@@ -2040,7 +2040,7 @@
         <v>หญิง</v>
       </c>
       <c r="I47" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J47" t="str">
         <v/>
@@ -2075,7 +2075,7 @@
         <v>หญิง</v>
       </c>
       <c r="I48" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J48" t="str">
         <v/>
@@ -2110,7 +2110,7 @@
         <v>หญิง</v>
       </c>
       <c r="I49" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J49" t="str">
         <v/>
@@ -2145,7 +2145,7 @@
         <v>ชาย</v>
       </c>
       <c r="I50" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J50" t="str">
         <v/>
@@ -2180,7 +2180,7 @@
         <v>ชาย</v>
       </c>
       <c r="I51" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J51" t="str">
         <v/>
@@ -2215,7 +2215,7 @@
         <v>ชาย</v>
       </c>
       <c r="I52" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J52" t="str">
         <v/>
@@ -2250,7 +2250,7 @@
         <v>ชาย</v>
       </c>
       <c r="I53" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J53" t="str">
         <v/>
@@ -2285,7 +2285,7 @@
         <v>หญิง</v>
       </c>
       <c r="I54" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J54" t="str">
         <v/>
@@ -2320,7 +2320,7 @@
         <v>หญิง</v>
       </c>
       <c r="I55" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J55" t="str">
         <v/>
@@ -2355,7 +2355,7 @@
         <v>หญิง</v>
       </c>
       <c r="I56" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J56" t="str">
         <v/>
@@ -2390,7 +2390,7 @@
         <v>ชาย</v>
       </c>
       <c r="I57" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J57" t="str">
         <v/>
@@ -2425,7 +2425,7 @@
         <v>ชาย</v>
       </c>
       <c r="I58" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J58" t="str">
         <v/>
@@ -2460,7 +2460,7 @@
         <v>หญิง</v>
       </c>
       <c r="I59" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J59" t="str">
         <v/>
@@ -2495,7 +2495,7 @@
         <v>หญิง</v>
       </c>
       <c r="I60" t="str">
-        <v>สแตนเชียร์, เชียร์ลีดเดอร์</v>
+        <v>ฝ่ายสแตนเชียร์, ฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J60" t="str">
         <v/>
@@ -2530,7 +2530,7 @@
         <v>หญิง</v>
       </c>
       <c r="I61" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J61" t="str">
         <v/>
@@ -2565,7 +2565,7 @@
         <v>หญิง</v>
       </c>
       <c r="I62" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J62" t="str">
         <v/>
@@ -2600,7 +2600,7 @@
         <v>ชาย</v>
       </c>
       <c r="I63" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J63" t="str">
         <v/>
@@ -2635,7 +2635,7 @@
         <v>ชาย</v>
       </c>
       <c r="I64" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J64" t="str">
         <v/>
@@ -2670,7 +2670,7 @@
         <v>ชาย</v>
       </c>
       <c r="I65" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J65" t="str">
         <v/>
@@ -2705,7 +2705,7 @@
         <v>ชาย</v>
       </c>
       <c r="I66" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J66" t="str">
         <v/>
@@ -2740,7 +2740,7 @@
         <v>หญิง</v>
       </c>
       <c r="I67" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J67" t="str">
         <v/>
@@ -2775,7 +2775,7 @@
         <v>ชาย</v>
       </c>
       <c r="I68" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J68" t="str">
         <v/>
@@ -2810,7 +2810,7 @@
         <v>ชาย</v>
       </c>
       <c r="I69" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J69" t="str">
         <v/>
@@ -2845,7 +2845,7 @@
         <v>ชาย</v>
       </c>
       <c r="I70" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J70" t="str">
         <v/>
@@ -2880,7 +2880,7 @@
         <v>หญิง</v>
       </c>
       <c r="I71" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J71" t="str">
         <v/>
@@ -2915,7 +2915,7 @@
         <v>หญิง</v>
       </c>
       <c r="I72" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J72" t="str">
         <v/>
@@ -2950,7 +2950,7 @@
         <v>ชาย</v>
       </c>
       <c r="I73" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -2985,7 +2985,7 @@
         <v>ชาย</v>
       </c>
       <c r="I74" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J74" t="str">
         <v/>
@@ -3020,7 +3020,7 @@
         <v>ชาย</v>
       </c>
       <c r="I75" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J75" t="str">
         <v/>
@@ -3055,7 +3055,7 @@
         <v>หญิง</v>
       </c>
       <c r="I76" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J76" t="str">
         <v/>
@@ -3090,7 +3090,7 @@
         <v>หญิง</v>
       </c>
       <c r="I77" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J77" t="str">
         <v/>
@@ -3125,7 +3125,7 @@
         <v>ชาย</v>
       </c>
       <c r="I78" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J78" t="str">
         <v/>
@@ -3160,7 +3160,7 @@
         <v>ชาย</v>
       </c>
       <c r="I79" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J79" t="str">
         <v/>
@@ -3195,7 +3195,7 @@
         <v>หญิง</v>
       </c>
       <c r="I80" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J80" t="str">
         <v/>
@@ -3230,7 +3230,7 @@
         <v>หญิง</v>
       </c>
       <c r="I81" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -3265,7 +3265,7 @@
         <v>หญิง</v>
       </c>
       <c r="I82" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J82" t="str">
         <v/>
@@ -3300,7 +3300,7 @@
         <v>ชาย</v>
       </c>
       <c r="I83" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J83" t="str">
         <v/>
@@ -3335,7 +3335,7 @@
         <v>ชาย</v>
       </c>
       <c r="I84" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J84" t="str">
         <v/>
@@ -3370,7 +3370,7 @@
         <v>หญิง</v>
       </c>
       <c r="I85" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J85" t="str">
         <v/>
@@ -3405,7 +3405,7 @@
         <v>หญิง</v>
       </c>
       <c r="I86" t="str">
-        <v>สแตนเชียร์</v>
+        <v>ฝ่ายสแตนเชียร์</v>
       </c>
       <c r="J86" t="str">
         <v/>
@@ -3591,7 +3591,7 @@
         <v>หญิง</v>
       </c>
       <c r="I5" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J5" t="str">
         <v>092-376-2675</v>
@@ -3626,7 +3626,7 @@
         <v>หญิง</v>
       </c>
       <c r="I6" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J6" t="str">
         <v>095-191-5990</v>
@@ -3696,7 +3696,7 @@
         <v>หญิง</v>
       </c>
       <c r="I8" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J8" t="str">
         <v>095-135-9335</v>
@@ -4116,7 +4116,7 @@
         <v>หญิง</v>
       </c>
       <c r="I20" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J20" t="str">
         <v>082-594-4531</v>
@@ -4151,7 +4151,7 @@
         <v>หญิง</v>
       </c>
       <c r="I21" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J21" t="str">
         <v>099-272-6458</v>
@@ -4606,7 +4606,7 @@
         <v>หญิง</v>
       </c>
       <c r="I34" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J34" t="str">
         <v>096-104-0004</v>
@@ -4886,7 +4886,7 @@
         <v>หญิง</v>
       </c>
       <c r="I42" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J42" t="str">
         <v>061-314-0692</v>
@@ -5306,7 +5306,7 @@
         <v>หญิง</v>
       </c>
       <c r="I54" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J54" t="str">
         <v>082-119-4569</v>
@@ -5376,7 +5376,7 @@
         <v>หญิง</v>
       </c>
       <c r="I56" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J56" t="str">
         <v>095-796-7899</v>
@@ -5411,7 +5411,7 @@
         <v>หญิง</v>
       </c>
       <c r="I57" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J57" t="str">
         <v>097-145-3589</v>
@@ -5481,7 +5481,7 @@
         <v>ชาย</v>
       </c>
       <c r="I59" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J59" t="str">
         <v>095-357-2991</v>
@@ -5551,7 +5551,7 @@
         <v>หญิง</v>
       </c>
       <c r="I61" t="str">
-        <v>ฟุตบอล, ขบวนพาเหรด</v>
+        <v>ฟุตบอล, ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J61" t="str">
         <v>091-030-4248</v>
@@ -5586,7 +5586,7 @@
         <v>หญิง</v>
       </c>
       <c r="I62" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J62" t="str">
         <v>094-006-5719</v>
@@ -5796,7 +5796,7 @@
         <v>ชาย</v>
       </c>
       <c r="I68" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J68" t="str">
         <v>096-962-5615</v>
@@ -5831,7 +5831,7 @@
         <v>ชาย</v>
       </c>
       <c r="I69" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J69" t="str">
         <v>084-967-9146</v>
@@ -5866,7 +5866,7 @@
         <v>หญิง</v>
       </c>
       <c r="I70" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J70" t="str">
         <v>098-819-6918</v>
@@ -5901,7 +5901,7 @@
         <v>หญิง</v>
       </c>
       <c r="I71" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J71" t="str">
         <v>082-591-2812</v>
@@ -5971,7 +5971,7 @@
         <v>ชาย</v>
       </c>
       <c r="I73" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J73" t="str">
         <v>096-765-6020</v>
@@ -6041,7 +6041,7 @@
         <v>ชาย</v>
       </c>
       <c r="I75" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J75" t="str">
         <v/>
@@ -6076,7 +6076,7 @@
         <v>หญิง</v>
       </c>
       <c r="I76" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J76" t="str">
         <v>098-384-5253</v>
@@ -6111,7 +6111,7 @@
         <v>หญิง</v>
       </c>
       <c r="I77" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J77" t="str">
         <v>064-326-1595</v>
@@ -6472,7 +6472,7 @@
         <v>หญิง</v>
       </c>
       <c r="I6" t="str">
-        <v>ดรัมเมเยอร์</v>
+        <v>ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J6" t="str">
         <v>099-616-9767</v>
@@ -6577,7 +6577,7 @@
         <v>หญิง</v>
       </c>
       <c r="I9" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J9" t="str">
         <v>091-049-3472</v>
@@ -6752,7 +6752,7 @@
         <v>หญิง</v>
       </c>
       <c r="I14" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J14" t="str">
         <v>083-097-3532</v>
@@ -6822,7 +6822,7 @@
         <v>หญิง</v>
       </c>
       <c r="I16" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J16" t="str">
         <v>099-738-2345</v>
@@ -6857,7 +6857,7 @@
         <v>หญิง</v>
       </c>
       <c r="I17" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J17" t="str">
         <v>098-738-9760</v>
@@ -6997,7 +6997,7 @@
         <v>หญิง</v>
       </c>
       <c r="I21" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J21" t="str">
         <v>096-294-5586</v>
@@ -7207,7 +7207,7 @@
         <v>หญิง</v>
       </c>
       <c r="I27" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J27" t="str">
         <v>082-965-5881</v>
@@ -7242,7 +7242,7 @@
         <v>หญิง</v>
       </c>
       <c r="I28" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J28" t="str">
         <v>083-097-3619</v>
@@ -7522,7 +7522,7 @@
         <v>หญิง</v>
       </c>
       <c r="I36" t="str">
-        <v>ดรัมเมเยอร์</v>
+        <v>ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J36" t="str">
         <v>085-849-9682</v>
@@ -7557,7 +7557,7 @@
         <v>หญิง</v>
       </c>
       <c r="I37" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J37" t="str">
         <v>063-019-1154</v>
@@ -7592,7 +7592,7 @@
         <v>หญิง</v>
       </c>
       <c r="I38" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J38" t="str">
         <v>098-689-7527</v>
@@ -7627,7 +7627,7 @@
         <v>หญิง</v>
       </c>
       <c r="I39" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J39" t="str">
         <v>065-250-6293</v>
@@ -7802,7 +7802,7 @@
         <v>หญิง</v>
       </c>
       <c r="I44" t="str">
-        <v>ดรัมเมเยอร์, ฟุตบอล</v>
+        <v>ฝ่ายดรัมเมเยอร์, ฟุตบอล</v>
       </c>
       <c r="J44" t="str">
         <v>080-800-6634</v>
@@ -7837,7 +7837,7 @@
         <v>หญิง</v>
       </c>
       <c r="I45" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J45" t="str">
         <v>062-226-3633</v>
@@ -8222,7 +8222,7 @@
         <v>หญิง</v>
       </c>
       <c r="I56" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J56" t="str">
         <v>095-358-9547</v>
@@ -8502,7 +8502,7 @@
         <v>หญิง</v>
       </c>
       <c r="I64" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J64" t="str">
         <v>065-975-1810</v>
@@ -8642,7 +8642,7 @@
         <v>หญิง</v>
       </c>
       <c r="I68" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J68" t="str">
         <v>096-084-2669</v>
@@ -8677,7 +8677,7 @@
         <v>หญิง</v>
       </c>
       <c r="I69" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J69" t="str">
         <v>080-137-4426</v>
@@ -8817,7 +8817,7 @@
         <v>หญิง</v>
       </c>
       <c r="I73" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J73" t="str">
         <v>098-951-4742</v>
@@ -8957,7 +8957,7 @@
         <v>หญิง</v>
       </c>
       <c r="I77" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J77" t="str">
         <v>092-825-3690</v>
@@ -9353,7 +9353,7 @@
         <v>หญิง</v>
       </c>
       <c r="I5" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J5" t="str">
         <v>090-494-0960</v>
@@ -9563,7 +9563,7 @@
         <v>หญิง</v>
       </c>
       <c r="I11" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J11" t="str">
         <v>083-337-9454</v>
@@ -9633,7 +9633,7 @@
         <v>หญิง</v>
       </c>
       <c r="I13" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J13" t="str">
         <v>061-230-7804</v>
@@ -9913,7 +9913,7 @@
         <v>หญิง</v>
       </c>
       <c r="I21" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J21" t="str">
         <v>098-463-4302</v>
@@ -10088,7 +10088,7 @@
         <v>หญิง</v>
       </c>
       <c r="I26" t="str">
-        <v>ฝ่ายเชียร์ลีดเดอร์, ขบวนพาเหรด</v>
+        <v>ฝ่ายเชียร์ลีดเดอร์, ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J26" t="str">
         <v>062-514-6471</v>
@@ -10123,7 +10123,7 @@
         <v>หญิง</v>
       </c>
       <c r="I27" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J27" t="str">
         <v>061-193-3676</v>
@@ -10298,7 +10298,7 @@
         <v>หญิง</v>
       </c>
       <c r="I32" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J32" t="str">
         <v>092-445-8482</v>
@@ -10403,7 +10403,7 @@
         <v>ชาย</v>
       </c>
       <c r="I35" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J35" t="str">
         <v>064-326-0371</v>
@@ -10438,7 +10438,7 @@
         <v>ชาย</v>
       </c>
       <c r="I36" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J36" t="str">
         <v>062-479-0695</v>
@@ -10473,7 +10473,7 @@
         <v>หญิง</v>
       </c>
       <c r="I37" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J37" t="str">
         <v>065-837-6263</v>
@@ -10508,7 +10508,7 @@
         <v>หญิง</v>
       </c>
       <c r="I38" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J38" t="str">
         <v>098-269-0466</v>
@@ -10543,7 +10543,7 @@
         <v>หญิง</v>
       </c>
       <c r="I39" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J39" t="str">
         <v>060-373-1209</v>
@@ -10613,7 +10613,7 @@
         <v>หญิง</v>
       </c>
       <c r="I41" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J41" t="str">
         <v>099-172-8992</v>
@@ -10788,7 +10788,7 @@
         <v>หญิง</v>
       </c>
       <c r="I46" t="str">
-        <v>สวัสดิการ</v>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J46" t="str">
         <v>083-799-7780</v>
@@ -10823,7 +10823,7 @@
         <v>หญิง</v>
       </c>
       <c r="I47" t="str">
-        <v>สวัสดิการ, วอลเลย์บอล, วิ่ง 16 ขา</v>
+        <v>ฝ่ายสวัสดิการ, วอลเลย์บอล, วิ่ง 16 ขา</v>
       </c>
       <c r="J47" t="str">
         <v>091-046-2589</v>
@@ -11068,7 +11068,7 @@
         <v>หญิง</v>
       </c>
       <c r="I54" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J54" t="str">
         <v>083-852-0626</v>
@@ -11208,7 +11208,7 @@
         <v>หญิง</v>
       </c>
       <c r="I58" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J58" t="str">
         <v>061-160-2991</v>
@@ -11628,7 +11628,7 @@
         <v>หญิง</v>
       </c>
       <c r="I70" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J70" t="str">
         <v>082-906-9603</v>
@@ -11663,7 +11663,7 @@
         <v>หญิง</v>
       </c>
       <c r="I71" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J71" t="str">
         <v>095-682-6677</v>
@@ -11698,7 +11698,7 @@
         <v>ชาย</v>
       </c>
       <c r="I72" t="str">
-        <v>วิ่ง 16 ขา, ขบวนพาเหรด</v>
+        <v>วิ่ง 16 ขา, ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J72" t="str">
         <v>096-663-3965</v>
@@ -11733,7 +11733,7 @@
         <v>ชาย</v>
       </c>
       <c r="I73" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J73" t="str">
         <v>096-664-4036</v>
@@ -11768,7 +11768,7 @@
         <v>ชาย</v>
       </c>
       <c r="I74" t="str">
-        <v>วิ่ง 16 ขา, ขบวนพาเหรด</v>
+        <v>วิ่ง 16 ขา, ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J74" t="str">
         <v>093-952-7843</v>
@@ -11803,7 +11803,7 @@
         <v>หญิง</v>
       </c>
       <c r="I75" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J75" t="str">
         <v>092-506-8497</v>
@@ -11838,7 +11838,7 @@
         <v>หญิง</v>
       </c>
       <c r="I76" t="str">
-        <v>ขบวนพาเหรด</v>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J76" t="str">
         <v>084-167-2074</v>
@@ -11943,7 +11943,7 @@
         <v>หญิง</v>
       </c>
       <c r="I79" t="str">
-        <v>ดรัมเมเยอร์</v>
+        <v>ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J79" t="str">
         <v>098-817-0691</v>
@@ -11978,7 +11978,7 @@
         <v>หญิง</v>
       </c>
       <c r="I80" t="str">
-        <v>ดรัมเมเยอร์</v>
+        <v>ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J80" t="str">
         <v>096-359-4382</v>
@@ -12118,7 +12118,7 @@
         <v>หญิง</v>
       </c>
       <c r="I84" t="str">
-        <v>อุปกรณ์และพร็อพ</v>
+        <v>ฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J84" t="str">
         <v>083-219-5152</v>
@@ -12339,7 +12339,7 @@
         <v>หญิง</v>
       </c>
       <c r="I5" t="str">
-        <v>สตาฟขบวนพาเหรด</v>
+        <v>สตาฟฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J5" t="str">
         <v>097-219-3314</v>
@@ -12409,7 +12409,7 @@
         <v>หญิง</v>
       </c>
       <c r="I7" t="str">
-        <v>คัลเลอร์การ์ด</v>
+        <v>ฝ่ายคัลเลอร์การ์ด</v>
       </c>
       <c r="J7" t="str">
         <v>063-786-4656</v>
@@ -12479,7 +12479,7 @@
         <v>ชาย</v>
       </c>
       <c r="I9" t="str">
-        <v>สตาฟอุปกรณ์และพร็อพ</v>
+        <v>สตาฟฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J9" t="str">
         <v>063-891-3857</v>
@@ -12549,7 +12549,7 @@
         <v>หญิง</v>
       </c>
       <c r="I11" t="str">
-        <v>สตาฟกองเชียร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J11" t="str">
         <v>062-220-7959</v>
@@ -12584,7 +12584,7 @@
         <v>หญิง</v>
       </c>
       <c r="I12" t="str">
-        <v>สตาฟกองเชียร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J12" t="str">
         <v>063-546-8896</v>
@@ -12689,7 +12689,7 @@
         <v>หญิง</v>
       </c>
       <c r="I15" t="str">
-        <v>สตาฟอุปกรณ์และพร็อพ</v>
+        <v>สตาฟฝ่ายอุปกรณ์และพร็อพ</v>
       </c>
       <c r="J15" t="str">
         <v>061-283-2615</v>
@@ -12864,7 +12864,7 @@
         <v>หญิง</v>
       </c>
       <c r="I20" t="str">
-        <v>สตาฟเชียร์ลีดเดอร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J20" t="str">
         <v>064-560-7577</v>
@@ -12934,7 +12934,7 @@
         <v>หญิง</v>
       </c>
       <c r="I22" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J22" t="str">
         <v>081-160-6764</v>
@@ -13109,7 +13109,7 @@
         <v>หญิง</v>
       </c>
       <c r="I27" t="str">
-        <v>ฟุตบอล, ดรัมเมเยอร์</v>
+        <v>ฟุตบอล, ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J27" t="str">
         <v>061-553-0691</v>
@@ -13144,7 +13144,7 @@
         <v>หญิง</v>
       </c>
       <c r="I28" t="str">
-        <v>ฟุตบอล, ดรัมเมเยอร์</v>
+        <v>ฟุตบอล, ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J28" t="str">
         <v>080-887-7109</v>
@@ -13214,7 +13214,7 @@
         <v>หญิง</v>
       </c>
       <c r="I30" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J30" t="str">
         <v>099-237-8944</v>
@@ -13249,7 +13249,7 @@
         <v>หญิง</v>
       </c>
       <c r="I31" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J31" t="str">
         <v>095-658-9660</v>
@@ -13424,7 +13424,7 @@
         <v>หญิง</v>
       </c>
       <c r="I36" t="str">
-        <v>หัวหน้าฝ่ายกองเชียร์</v>
+        <v>หัวหน้าฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J36" t="str">
         <v>065-493-0315</v>
@@ -13459,7 +13459,7 @@
         <v>หญิง</v>
       </c>
       <c r="I37" t="str">
-        <v>สตาฟขบวนพาเหรด</v>
+        <v>สตาฟฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J37" t="str">
         <v/>
@@ -13494,7 +13494,7 @@
         <v>หญิง</v>
       </c>
       <c r="I38" t="str">
-        <v>หัวหน้าฝ่ายกองเชียร์</v>
+        <v>หัวหน้าฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J38" t="str">
         <v>083-884-2697</v>
@@ -13599,7 +13599,7 @@
         <v>หญิง</v>
       </c>
       <c r="I41" t="str">
-        <v>สตาฟเชียร์ลีดเดอร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J41" t="str">
         <v>080-736-1039</v>
@@ -13669,7 +13669,7 @@
         <v>หญิง</v>
       </c>
       <c r="I43" t="str">
-        <v>ดรัมเมเยอร์</v>
+        <v>ฝ่ายดรัมเมเยอร์</v>
       </c>
       <c r="J43" t="str">
         <v>099-263-2316</v>
@@ -13739,7 +13739,7 @@
         <v>หญิง</v>
       </c>
       <c r="I45" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J45" t="str">
         <v>065-678-3202</v>
@@ -13844,7 +13844,7 @@
         <v>หญิง</v>
       </c>
       <c r="I48" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J48" t="str">
         <v>065-291-7532</v>
@@ -13914,7 +13914,7 @@
         <v>หญิง</v>
       </c>
       <c r="I50" t="str">
-        <v>คัลเลอร์การ์ด</v>
+        <v>ฝ่ายคัลเลอร์การ์ด</v>
       </c>
       <c r="J50" t="str">
         <v/>
@@ -14019,7 +14019,7 @@
         <v>ชาย</v>
       </c>
       <c r="I53" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J53" t="str">
         <v>082-035-6213</v>
@@ -14194,7 +14194,7 @@
         <v>หญิง</v>
       </c>
       <c r="I58" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J58" t="str">
         <v>064-869-4386</v>
@@ -14264,7 +14264,7 @@
         <v>หญิง</v>
       </c>
       <c r="I60" t="str">
-        <v>สตาฟกองเชียร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J60" t="str">
         <v>065-687-9600</v>
@@ -14334,7 +14334,7 @@
         <v>หญิง</v>
       </c>
       <c r="I62" t="str">
-        <v>สตาฟกองเชียร์</v>
+        <v>สตาฟฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J62" t="str">
         <v>083-025-2578</v>
@@ -14544,7 +14544,7 @@
         <v>ชาย</v>
       </c>
       <c r="I68" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J68" t="str">
         <v>080-825-7625</v>
@@ -14719,7 +14719,7 @@
         <v>ชาย</v>
       </c>
       <c r="I73" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -14929,7 +14929,7 @@
         <v>ชาย</v>
       </c>
       <c r="I79" t="str">
-        <v>สตาฟสวัสดิการ</v>
+        <v>สตาฟฝ่ายสวัสดิการ</v>
       </c>
       <c r="J79" t="str">
         <v>091-969-6155</v>
@@ -14999,7 +14999,7 @@
         <v>หญิง</v>
       </c>
       <c r="I81" t="str">
-        <v>คัลเลอร์การ์ด</v>
+        <v>ฝ่ายคัลเลอร์การ์ด</v>
       </c>
       <c r="J81" t="str">
         <v/>

</xml_diff>

<commit_message>
Data: Fix missing student records for Veeraphat Moolchai (33629) and Thanaporn Chaiyameungcheun (32138)
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
@@ -6425,16 +6425,16 @@
         <v>ม.3/1</v>
       </c>
       <c r="E5">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F5" t="str">
-        <v>34049</v>
+        <v>33629</v>
       </c>
       <c r="G5" t="str">
-        <v>เด็กหญิงพชรพร รอดสุด</v>
+        <v>นายวีรภัทร มูลชัย</v>
       </c>
       <c r="H5" t="str">
-        <v>หญิง</v>
+        <v>ชาย</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -15138,16 +15138,16 @@
         <v>ม.6/1</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F4" t="str">
-        <v>32128</v>
+        <v>32138</v>
       </c>
       <c r="G4" t="str">
-        <v>นายภูมินทร์ หลวงแสง</v>
+        <v>นางสาวธนาภรณ์ ไชยเมืองชื่น</v>
       </c>
       <c r="H4" t="str">
-        <v>ชาย</v>
+        <v>หญิง</v>
       </c>
       <c r="I4" t="str">
         <v/>

</xml_diff>

<commit_message>
Sync: Pull latest Google Sheets roster, duties, and phone numbers into local JSON and Excel
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/รายชื่อคณะสีแสด_ปี69.xlsx
@@ -3661,10 +3661,10 @@
         <v>หญิง</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>เปตอง</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>098-567-1827</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -3766,10 +3766,10 @@
         <v>ชาย</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>080-747-3184</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -3836,10 +3836,10 @@
         <v>หญิง</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>095-389-8605</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -3871,7 +3871,7 @@
         <v>หญิง</v>
       </c>
       <c r="I13" t="str">
-        <v>วอลเลย์บอล</v>
+        <v>วอลเลย์บอล, ฟุตบอล</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -3941,7 +3941,7 @@
         <v>หญิง</v>
       </c>
       <c r="I15" t="str">
-        <v>วอลเลย์บอล</v>
+        <v>วอลเลย์บอล, ฟุตบอล</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -4361,10 +4361,10 @@
         <v>หญิง</v>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>064-251-9806</v>
       </c>
       <c r="K27" t="str">
         <v/>
@@ -4396,10 +4396,10 @@
         <v>หญิง</v>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>083-451-7140</v>
       </c>
       <c r="K28" t="str">
         <v/>
@@ -4431,10 +4431,10 @@
         <v>หญิง</v>
       </c>
       <c r="I29" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>065-858-8204</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -4641,10 +4641,10 @@
         <v>หญิง</v>
       </c>
       <c r="I35" t="str">
-        <v/>
+        <v>คัลเลอร์การ์ด</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>093-243-6307</v>
       </c>
       <c r="K35" t="str">
         <v/>
@@ -4663,7 +4663,7 @@
       <c r="D36" t="str">
         <v>ม.2/5</v>
       </c>
-      <c r="E36" t="str">
+      <c r="E36">
         <v>-</v>
       </c>
       <c r="F36" t="str">
@@ -4851,10 +4851,10 @@
         <v>หญิง</v>
       </c>
       <c r="I41" t="str">
-        <v/>
+        <v>ฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>093-393-1626</v>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -4921,10 +4921,10 @@
         <v>ชาย</v>
       </c>
       <c r="I43" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>091-027-7059</v>
       </c>
       <c r="K43" t="str">
         <v/>
@@ -5026,10 +5026,10 @@
         <v>หญิง</v>
       </c>
       <c r="I46" t="str">
-        <v/>
+        <v>ฝ่ายคัลเลอร์การ์ด</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>091-024-8039</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -5131,10 +5131,10 @@
         <v>หญิง</v>
       </c>
       <c r="I49" t="str">
-        <v/>
+        <v>คัลเลอร์การ์ด</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>065-379-1693</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -5236,10 +5236,10 @@
         <v>ชาย</v>
       </c>
       <c r="I52" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>080-854-1169</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -5341,10 +5341,10 @@
         <v>หญิง</v>
       </c>
       <c r="I55" t="str">
-        <v/>
+        <v>ฝ่ายเชียร์ลีดเดอร์</v>
       </c>
       <c r="J55" t="str">
-        <v/>
+        <v>061-794-0872</v>
       </c>
       <c r="K55" t="str">
         <v/>
@@ -5446,10 +5446,10 @@
         <v>ชาย</v>
       </c>
       <c r="I58" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J58" t="str">
-        <v/>
+        <v>081-077-9340</v>
       </c>
       <c r="K58" t="str">
         <v/>
@@ -6507,10 +6507,10 @@
         <v>หญิง</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>096-682-1854</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -6542,10 +6542,10 @@
         <v>หญิง</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>084-017-6210</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -7032,7 +7032,7 @@
         <v>หญิง</v>
       </c>
       <c r="I22" t="str">
-        <v>ฟุตบอล</v>
+        <v>ฟุตบอล, กรีฑา, บาสเกตบอล</v>
       </c>
       <c r="J22" t="str">
         <v>061-983-7797</v>
@@ -7697,10 +7697,10 @@
         <v>ชาย</v>
       </c>
       <c r="I41" t="str">
-        <v/>
+        <v>กรีฑา</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>061-439-7907</v>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -7732,10 +7732,10 @@
         <v>หญิง</v>
       </c>
       <c r="I42" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>092-452-1062</v>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -7767,7 +7767,7 @@
         <v>หญิง</v>
       </c>
       <c r="I43" t="str">
-        <v>ฟุตบอล</v>
+        <v>ฟุตบอล, กรีฑา, บาสเกตบอล</v>
       </c>
       <c r="J43" t="str">
         <v>093-131-8108</v>
@@ -8047,10 +8047,10 @@
         <v>หญิง</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>082-086-7639</v>
       </c>
       <c r="K51" t="str">
         <v/>
@@ -8747,10 +8747,10 @@
         <v>ชาย</v>
       </c>
       <c r="I71" t="str">
-        <v/>
+        <v>ฟุตบอล</v>
       </c>
       <c r="J71" t="str">
-        <v/>
+        <v>061-150-8435</v>
       </c>
       <c r="K71" t="str">
         <v/>
@@ -9388,10 +9388,10 @@
         <v>หญิง</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>088-599-5886</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -9423,10 +9423,10 @@
         <v>หญิง</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>063-035-2452</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -9843,10 +9843,10 @@
         <v>หญิง</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>084-049-5162</v>
       </c>
       <c r="K19" t="str">
         <v/>
@@ -9878,10 +9878,10 @@
         <v>หญิง</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>063-751-0224</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -9948,10 +9948,10 @@
         <v>ชาย</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>062-120-5203</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -10053,10 +10053,10 @@
         <v>หญิง</v>
       </c>
       <c r="I25" t="str">
-        <v/>
+        <v>คัลเลอร์การ์ด, ฝ่ายคัลเลอร์การ์ด</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>065-484-2530</v>
       </c>
       <c r="K25" t="str">
         <v/>
@@ -10158,10 +10158,10 @@
         <v>ชาย</v>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>064-591-4070</v>
       </c>
       <c r="K28" t="str">
         <v/>
@@ -10228,10 +10228,10 @@
         <v>ชาย</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>วิ่ง 16 ขา</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>099-435-6995</v>
       </c>
       <c r="K30" t="str">
         <v/>
@@ -10263,10 +10263,10 @@
         <v>หญิง</v>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>คัลเลอร์การ์ด</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>094-920-3178</v>
       </c>
       <c r="K31" t="str">
         <v/>
@@ -10648,10 +10648,10 @@
         <v>ชาย</v>
       </c>
       <c r="I42" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>095-602-8523</v>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -10718,10 +10718,10 @@
         <v>หญิง</v>
       </c>
       <c r="I44" t="str">
-        <v/>
+        <v>ฟุตบอล</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>099-193-7702</v>
       </c>
       <c r="K44" t="str">
         <v/>
@@ -10963,10 +10963,10 @@
         <v>ชาย</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>วิ่ง 16 ขา</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>083-214-0843</v>
       </c>
       <c r="K51" t="str">
         <v/>
@@ -11173,10 +11173,10 @@
         <v>หญิง</v>
       </c>
       <c r="I57" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J57" t="str">
-        <v/>
+        <v>098-749-3595</v>
       </c>
       <c r="K57" t="str">
         <v/>
@@ -11265,7 +11265,7 @@
       <c r="D60" t="str">
         <v>ม.4/9</v>
       </c>
-      <c r="E60" t="str">
+      <c r="E60">
         <v>-</v>
       </c>
       <c r="F60" t="str">
@@ -11300,7 +11300,7 @@
       <c r="D61" t="str">
         <v>ม.4/9</v>
       </c>
-      <c r="E61" t="str">
+      <c r="E61">
         <v>-</v>
       </c>
       <c r="F61" t="str">
@@ -11418,10 +11418,10 @@
         <v>หญิง</v>
       </c>
       <c r="I64" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J64" t="str">
-        <v/>
+        <v>093-132-7524</v>
       </c>
       <c r="K64" t="str">
         <v/>
@@ -11453,10 +11453,10 @@
         <v>หญิง</v>
       </c>
       <c r="I65" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J65" t="str">
-        <v/>
+        <v>095-635-3078</v>
       </c>
       <c r="K65" t="str">
         <v/>
@@ -11488,10 +11488,10 @@
         <v>หญิง</v>
       </c>
       <c r="I66" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J66" t="str">
-        <v/>
+        <v>098-721-9619</v>
       </c>
       <c r="K66" t="str">
         <v/>
@@ -11558,10 +11558,10 @@
         <v>ชาย</v>
       </c>
       <c r="I68" t="str">
-        <v/>
+        <v>ฝ่ายพร็อพ</v>
       </c>
       <c r="J68" t="str">
-        <v/>
+        <v>084-050-3337</v>
       </c>
       <c r="K68" t="str">
         <v/>
@@ -11873,10 +11873,10 @@
         <v>ชาย</v>
       </c>
       <c r="I77" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J77" t="str">
-        <v/>
+        <v>061-269-5726</v>
       </c>
       <c r="K77" t="str">
         <v/>
@@ -11908,10 +11908,10 @@
         <v>ชาย</v>
       </c>
       <c r="I78" t="str">
-        <v/>
+        <v>ฝ่ายสวัสดิการ</v>
       </c>
       <c r="J78" t="str">
-        <v/>
+        <v>096-667-3887</v>
       </c>
       <c r="K78" t="str">
         <v/>
@@ -12013,7 +12013,7 @@
         <v>หญิง</v>
       </c>
       <c r="I81" t="str">
-        <v/>
+        <v>คัลเลอร์การ์ด</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -12724,7 +12724,7 @@
         <v>ชาย</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>กรีฑา</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -12956,7 +12956,7 @@
       <c r="D23" t="str">
         <v>ม.5/3</v>
       </c>
-      <c r="E23" t="str">
+      <c r="E23">
         <v>-</v>
       </c>
       <c r="F23" t="str">
@@ -13354,10 +13354,10 @@
         <v>ชาย</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>สตาฟเปตอง</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>096-976-2786</v>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -13879,10 +13879,10 @@
         <v>หญิง</v>
       </c>
       <c r="I49" t="str">
-        <v/>
+        <v>สตาฟฝ่ายพร็อพ</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>666-207-6517</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -13949,10 +13949,10 @@
         <v>หญิง</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>สตาฟฝ่ายพร็อพ</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>061-684-3615</v>
       </c>
       <c r="K51" t="str">
         <v/>
@@ -14054,10 +14054,10 @@
         <v>ชาย</v>
       </c>
       <c r="I54" t="str">
-        <v/>
+        <v>สตาฟฝ่ายพร็อพ</v>
       </c>
       <c r="J54" t="str">
-        <v/>
+        <v>083-214-8508</v>
       </c>
       <c r="K54" t="str">
         <v/>
@@ -14124,7 +14124,7 @@
         <v>หญิง</v>
       </c>
       <c r="I56" t="str">
-        <v/>
+        <v>ขบวนพาเหรด</v>
       </c>
       <c r="J56" t="str">
         <v/>
@@ -15605,10 +15605,10 @@
         <v>ชาย</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>บาสเกตบอล</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>082-590-6971</v>
       </c>
       <c r="K17" t="str">
         <v/>
@@ -17495,10 +17495,10 @@
         <v>หญิง</v>
       </c>
       <c r="I71" t="str">
-        <v/>
+        <v>ฝ่ายขบวนพาเหรด</v>
       </c>
       <c r="J71" t="str">
-        <v/>
+        <v>097-021-8357</v>
       </c>
       <c r="K71" t="str">
         <v/>

</xml_diff>